<commit_message>
Update Objective and co-benefits vocabularies, re-judge NFPP Objective, record bond framework exclusion
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inputs/template_en.xlsx
+++ b/inputs/template_en.xlsx
@@ -6196,7 +6196,7 @@
       </c>
       <c r="E12" s="449" t="inlineStr">
         <is>
-          <t>Climate change mitigation; Non-fossil energy; Energy efficiency; Green economy; Technological innovation; Energy security; Pollution control; Ecological protection; Circular economy; Adaptation; Green finance; Electrification; Industrial development; Green consumption; Information disclosure; Public awareness; Ozone layer protection</t>
+          <t>Climate change mitigation; Non-fossil energy; Energy efficiency; Green economy; Technological innovation; Energy security; Pollution control; Ecological protection; Biodiversity protection; Natural resource protection; Circular economy; Climate change adaptation; Green finance; Electrification; Industrial development; Green consumption; Information disclosure; Public awareness; Ozone layer protection</t>
         </is>
       </c>
       <c r="F12" s="459" t="n"/>
@@ -7500,7 +7500,7 @@
       </c>
       <c r="E46" s="449" t="inlineStr">
         <is>
-          <t>Adaptation; Air pollution; Energy supply security; Technological innovation; Poverty reduction; Employment; Industrial development; Other (non-exhaustive list, current options here based on IPCC)</t>
+          <t>Energy conservation; Technological innovation; Energy security; Pollution control; Ecological protection; Resource conservation; Circular economy; Renewable energy development; Public health; Climate change adaptation; Employment and poverty reduction; Industrial development; Biodiversity conservation; Desertification control; Green consumption; Food security</t>
         </is>
       </c>
       <c r="F46" s="459" t="n"/>

</xml_diff>